<commit_message>
Update Tâm Vet 2
</commit_message>
<xml_diff>
--- a/public/data/tamvet_product.xlsx
+++ b/public/data/tamvet_product.xlsx
@@ -19,7 +19,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="5">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -29,46 +29,17 @@
     </font>
     <font>
       <b val="1"/>
-      <color rgb="00FFFFFF"/>
     </font>
-    <font>
-      <b val="1"/>
-      <sz val="14"/>
-    </font>
-    <font>
-      <b val="1"/>
-      <color rgb="00FFFFFF"/>
-      <sz val="14"/>
-    </font>
-    <font/>
   </fonts>
-  <fills count="5">
+  <fills count="2">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00366092"/>
-        <bgColor rgb="00366092"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="0092D050"/>
-        <bgColor rgb="0092D050"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00C00000"/>
-        <bgColor rgb="00C00000"/>
-      </patternFill>
-    </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -76,29 +47,20 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -465,37 +427,10 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Y4"/>
+  <dimension ref="A1:Z4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="12" customWidth="1" min="1" max="1"/>
-    <col width="20" customWidth="1" min="2" max="2"/>
-    <col width="20" customWidth="1" min="3" max="3"/>
-    <col width="18" customWidth="1" min="4" max="4"/>
-    <col width="18" customWidth="1" min="5" max="5"/>
-    <col width="18" customWidth="1" min="6" max="6"/>
-    <col width="18" customWidth="1" min="7" max="7"/>
-    <col width="20" customWidth="1" min="8" max="8"/>
-    <col width="18" customWidth="1" min="9" max="9"/>
-    <col width="18" customWidth="1" min="10" max="10"/>
-    <col width="18" customWidth="1" min="11" max="11"/>
-    <col width="18" customWidth="1" min="12" max="12"/>
-    <col width="18" customWidth="1" min="13" max="13"/>
-    <col width="18" customWidth="1" min="14" max="14"/>
-    <col width="18" customWidth="1" min="15" max="15"/>
-    <col width="18" customWidth="1" min="16" max="16"/>
-    <col width="18" customWidth="1" min="17" max="17"/>
-    <col width="18" customWidth="1" min="18" max="18"/>
-    <col width="18" customWidth="1" min="19" max="19"/>
-    <col width="18" customWidth="1" min="20" max="20"/>
-    <col width="18" customWidth="1" min="21" max="21"/>
-    <col width="18" customWidth="1" min="22" max="22"/>
-    <col width="18" customWidth="1" min="23" max="23"/>
-    <col width="18" customWidth="1" min="24" max="24"/>
-    <col width="18" customWidth="1" min="25" max="25"/>
-  </cols>
   <sheetData>
-    <row r="1" ht="25" customHeight="1">
+    <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
           <t>id</t>
@@ -621,355 +556,359 @@
           <t>functions</t>
         </is>
       </c>
+      <c r="Z1" s="1" t="inlineStr">
+        <is>
+          <t>images</t>
+        </is>
+      </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="inlineStr">
+      <c r="A2" t="inlineStr">
         <is>
           <t>TAMVET001</t>
         </is>
       </c>
-      <c r="B2" s="2" t="inlineStr">
-        <is>
-          <t>Thuốc Kháng Sinh Amoxicillin 500mg</t>
-        </is>
-      </c>
-      <c r="C2" s="2" t="inlineStr">
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Thuốc Kháng Sinh Amoxicillin 500mg 2</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
         <is>
           <t>Thuốc Thú Cưng</t>
         </is>
       </c>
-      <c r="D2" s="2" t="n">
+      <c r="D2" t="n">
         <v>45000</v>
       </c>
-      <c r="E2" s="2" t="n">
+      <c r="E2" t="n">
         <v>50000</v>
       </c>
-      <c r="F2" s="2" t="inlineStr">
+      <c r="F2" t="inlineStr">
         <is>
           <t>Thuốc kháng sinh hiệu quả điều trị các bệnh nhiễm khuẩn</t>
         </is>
       </c>
-      <c r="G2" s="2" t="inlineStr">
-        <is>
-          <t>Amoxicillin 500mg là thuốc kháng sinh beta-lactam có hiệu quả cao trong điều trị các bệnh nhiễm khuẩn ở động vật.</t>
-        </is>
-      </c>
-      <c r="H2" s="2" t="inlineStr">
-        <is>
-          <t>/images/products/amoxicillin.jpg</t>
-        </is>
-      </c>
-      <c r="I2" s="2" t="inlineStr">
-        <is>
-          <t>TRUE</t>
-        </is>
-      </c>
-      <c r="J2" s="2" t="inlineStr">
-        <is>
-          <t>TRUE</t>
-        </is>
-      </c>
-      <c r="K2" s="2" t="inlineStr">
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>Amoxicillin 500mg là thuốc kháng sinh beta-lactam có hiệu quả cao trong điều trị các bệnh nhiễm khuẩn ở động vật.&lt;div&gt;&lt;b&gt;Kiểm tra chi tiết sản phẩm&lt;/b&gt;&lt;/div&gt;</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>/images/tamvet-85766dd7-1765992017.jpg</t>
+        </is>
+      </c>
+      <c r="I2" t="b">
+        <v>1</v>
+      </c>
+      <c r="J2" t="b">
+        <v>1</v>
+      </c>
+      <c r="K2" t="inlineStr">
         <is>
           <t>10 vỉ/hộp</t>
         </is>
       </c>
-      <c r="L2" s="2" t="n">
+      <c r="L2" t="n">
         <v>150</v>
       </c>
-      <c r="M2" s="2" t="inlineStr">
+      <c r="M2" t="inlineStr">
         <is>
           <t>Chó, Mèo, Gia súc</t>
         </is>
       </c>
-      <c r="N2" s="2" t="inlineStr">
+      <c r="N2" t="inlineStr">
         <is>
           <t>Tâm Vet</t>
         </is>
       </c>
-      <c r="O2" s="2" t="inlineStr">
+      <c r="O2" t="inlineStr">
         <is>
           <t>Việt Nam</t>
         </is>
       </c>
-      <c r="P2" s="2" t="inlineStr">
+      <c r="P2" t="inlineStr">
         <is>
           <t>VN123456</t>
         </is>
       </c>
-      <c r="Q2" s="2" t="inlineStr">
+      <c r="Q2" t="inlineStr">
         <is>
           <t>Amoxicillin trihydrate 500mg</t>
         </is>
       </c>
-      <c r="R2" s="2" t="inlineStr">
+      <c r="R2" t="inlineStr">
         <is>
           <t>Chó: 20-40mg/kg, Mèo: 15-25mg/kg</t>
         </is>
       </c>
-      <c r="S2" s="2" t="inlineStr">
+      <c r="S2" t="inlineStr">
         <is>
           <t>Uống sau ăn 2-3 lần/ngày</t>
         </is>
       </c>
-      <c r="T2" s="2" t="inlineStr">
+      <c r="T2" t="inlineStr">
         <is>
           <t>Không sử dụng với thú có dị ứng penicillin</t>
         </is>
       </c>
-      <c r="U2" s="2" t="inlineStr">
+      <c r="U2" t="inlineStr">
         <is>
           <t>Bảo quản nơi khô ráo, nhiệt độ 15-25°C</t>
         </is>
       </c>
-      <c r="V2" s="2" t="n">
+      <c r="V2" t="n">
         <v>4.5</v>
       </c>
-      <c r="W2" s="2" t="n">
+      <c r="W2" t="n">
         <v>32</v>
       </c>
-      <c r="X2" s="2" t="inlineStr">
+      <c r="X2" t="inlineStr">
         <is>
           <t>kháng sinh;nhiễm khuẩn;chó;mèo</t>
         </is>
       </c>
-      <c r="Y2" s="2" t="inlineStr">
+      <c r="Y2" t="inlineStr">
         <is>
           <t>Kháng khuẩn;Diệt vi khuẩn</t>
         </is>
       </c>
+      <c r="Z2" t="inlineStr"/>
     </row>
     <row r="3">
-      <c r="A3" s="2" t="inlineStr">
+      <c r="A3" t="inlineStr">
         <is>
           <t>TAMVET002</t>
         </is>
       </c>
-      <c r="B3" s="2" t="inlineStr">
+      <c r="B3" t="inlineStr">
         <is>
           <t>Vitamin B Complex Cho Gia Súc</t>
         </is>
       </c>
-      <c r="C3" s="2" t="inlineStr">
+      <c r="C3" t="inlineStr">
         <is>
           <t>Vitamin &amp; Thực Phẩm Chức Năng</t>
         </is>
       </c>
-      <c r="D3" s="2" t="n">
+      <c r="D3" t="n">
         <v>65000</v>
       </c>
-      <c r="E3" s="2" t="n">
+      <c r="E3" t="n">
         <v>75000</v>
       </c>
-      <c r="F3" s="2" t="inlineStr">
+      <c r="F3" t="inlineStr">
         <is>
           <t>Bổ sung vitamin B giúp tăng sức đề kháng cho gia súc</t>
         </is>
       </c>
-      <c r="G3" s="2" t="inlineStr">
+      <c r="G3" t="inlineStr">
         <is>
           <t>Vitamin B Complex là một sản phẩm bổ sung vitamin nhóm B toàn diện, giúp cải thiện sức khỏe tổng thể.</t>
         </is>
       </c>
-      <c r="H3" s="2" t="inlineStr">
+      <c r="H3" t="inlineStr">
         <is>
           <t>/images/products/vitamin-b.jpg</t>
         </is>
       </c>
-      <c r="I3" s="2" t="inlineStr">
-        <is>
-          <t>TRUE</t>
-        </is>
-      </c>
-      <c r="J3" s="2" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
-      </c>
-      <c r="K3" s="2" t="inlineStr">
+      <c r="I3" t="b">
+        <v>1</v>
+      </c>
+      <c r="J3" t="b">
+        <v>0</v>
+      </c>
+      <c r="K3" t="inlineStr">
         <is>
           <t>100ml/chai</t>
         </is>
       </c>
-      <c r="L3" s="2" t="n">
+      <c r="L3" t="n">
         <v>200</v>
       </c>
-      <c r="M3" s="2" t="inlineStr">
+      <c r="M3" t="inlineStr">
         <is>
           <t>Gia súc</t>
         </is>
       </c>
-      <c r="N3" s="2" t="inlineStr">
+      <c r="N3" t="inlineStr">
         <is>
           <t>Tâm Vet</t>
         </is>
       </c>
-      <c r="O3" s="2" t="inlineStr">
+      <c r="O3" t="inlineStr">
         <is>
           <t>Việt Nam</t>
         </is>
       </c>
-      <c r="P3" s="2" t="inlineStr">
+      <c r="P3" t="inlineStr">
         <is>
           <t>VN123457</t>
         </is>
       </c>
-      <c r="Q3" s="2" t="inlineStr">
+      <c r="Q3" t="inlineStr">
         <is>
           <t>Thiamine,Riboflavin,Niacin,Pyridoxine</t>
         </is>
       </c>
-      <c r="R3" s="2" t="inlineStr">
+      <c r="R3" t="inlineStr">
         <is>
           <t>5-10ml/ngày/đầu gia súc</t>
         </is>
       </c>
-      <c r="S3" s="2" t="inlineStr">
+      <c r="S3" t="inlineStr">
         <is>
           <t>Trộn vào thức ăn hoặc cho uống trực tiếp</t>
         </is>
       </c>
-      <c r="T3" s="2" t="inlineStr">
+      <c r="T3" t="inlineStr">
         <is>
           <t>Bảo quản trong nơi mát mẻ, tránh ánh sáng</t>
         </is>
       </c>
-      <c r="U3" s="2" t="inlineStr">
+      <c r="U3" t="inlineStr">
         <is>
           <t>Bảo quản ở 2-8°C</t>
         </is>
       </c>
-      <c r="V3" s="2" t="n">
+      <c r="V3" t="n">
         <v>4.2</v>
       </c>
-      <c r="W3" s="2" t="n">
+      <c r="W3" t="n">
         <v>18</v>
       </c>
-      <c r="X3" s="2" t="inlineStr">
+      <c r="X3" t="inlineStr">
         <is>
           <t>vitamin;bổ sung;gia súc</t>
         </is>
       </c>
-      <c r="Y3" s="2" t="inlineStr">
+      <c r="Y3" t="inlineStr">
         <is>
           <t>Tăng sức đề kháng;Cải thiện sức khỏe</t>
         </is>
       </c>
+      <c r="Z3" t="inlineStr">
+        <is>
+          <t>n</t>
+        </is>
+      </c>
     </row>
     <row r="4">
-      <c r="A4" s="2" t="inlineStr">
+      <c r="A4" t="inlineStr">
         <is>
           <t>TAMVET003</t>
         </is>
       </c>
-      <c r="B4" s="2" t="inlineStr">
+      <c r="B4" t="inlineStr">
         <is>
           <t>Chế Phẩm Vi Sinh Tăng Tiêu Hóa</t>
         </is>
       </c>
-      <c r="C4" s="2" t="inlineStr">
+      <c r="C4" t="inlineStr">
         <is>
           <t>Chế Phẩm Sinh Học</t>
         </is>
       </c>
-      <c r="D4" s="2" t="n">
+      <c r="D4" t="n">
         <v>85000</v>
       </c>
-      <c r="E4" s="2" t="n">
+      <c r="E4" t="n">
         <v>95000</v>
       </c>
-      <c r="F4" s="2" t="inlineStr">
+      <c r="F4" t="inlineStr">
         <is>
           <t>Chế phẩm vi sinh giúp cân bằng hệ tiêu hóa</t>
         </is>
       </c>
-      <c r="G4" s="2" t="inlineStr">
+      <c r="G4" t="inlineStr">
         <is>
           <t>Chế phẩm này chứa các chủng vi sinh lợi ích giúp cân bằng hệ vi sinh đường ruột.</t>
         </is>
       </c>
-      <c r="H4" s="2" t="inlineStr">
+      <c r="H4" t="inlineStr">
         <is>
           <t>/images/products/probiotic.jpg</t>
         </is>
       </c>
-      <c r="I4" s="2" t="inlineStr">
-        <is>
-          <t>TRUE</t>
-        </is>
-      </c>
-      <c r="J4" s="2" t="inlineStr">
-        <is>
-          <t>TRUE</t>
-        </is>
-      </c>
-      <c r="K4" s="2" t="inlineStr">
+      <c r="I4" t="b">
+        <v>1</v>
+      </c>
+      <c r="J4" t="b">
+        <v>1</v>
+      </c>
+      <c r="K4" t="inlineStr">
         <is>
           <t>500g/kg</t>
         </is>
       </c>
-      <c r="L4" s="2" t="n">
+      <c r="L4" t="n">
         <v>120</v>
       </c>
-      <c r="M4" s="2" t="inlineStr">
+      <c r="M4" t="inlineStr">
         <is>
           <t>Gia cầm, Gia súc, Cá</t>
         </is>
       </c>
-      <c r="N4" s="2" t="inlineStr">
+      <c r="N4" t="inlineStr">
         <is>
           <t>Tâm Vet</t>
         </is>
       </c>
-      <c r="O4" s="2" t="inlineStr">
+      <c r="O4" t="inlineStr">
         <is>
           <t>Việt Nam</t>
         </is>
       </c>
-      <c r="P4" s="2" t="inlineStr">
+      <c r="P4" t="inlineStr">
         <is>
           <t>VN123458</t>
         </is>
       </c>
-      <c r="Q4" s="2" t="inlineStr">
+      <c r="Q4" t="inlineStr">
         <is>
           <t>Bacillus subtilis,Lactobacillus,Bifidobacterium</t>
         </is>
       </c>
-      <c r="R4" s="2" t="inlineStr">
+      <c r="R4" t="inlineStr">
         <is>
           <t>5-10g/tấn thức ăn</t>
         </is>
       </c>
-      <c r="S4" s="2" t="inlineStr">
+      <c r="S4" t="inlineStr">
         <is>
           <t>Trộn đều vào thức ăn tươi</t>
         </is>
       </c>
-      <c r="T4" s="2" t="inlineStr">
+      <c r="T4" t="inlineStr">
         <is>
           <t>Bảo quản ở nhiệt độ thấp, tránh ẩm ướt</t>
         </is>
       </c>
-      <c r="U4" s="2" t="inlineStr">
+      <c r="U4" t="inlineStr">
         <is>
           <t>Bảo quản ở 2-8°C hoặc -18°C</t>
         </is>
       </c>
-      <c r="V4" s="2" t="n">
+      <c r="V4" t="n">
         <v>4.8</v>
       </c>
-      <c r="W4" s="2" t="n">
+      <c r="W4" t="n">
         <v>45</v>
       </c>
-      <c r="X4" s="2" t="inlineStr">
+      <c r="X4" t="inlineStr">
         <is>
           <t>vi sinh;tiêu hóa;chế phẩm</t>
         </is>
       </c>
-      <c r="Y4" s="2" t="inlineStr">
+      <c r="Y4" t="inlineStr">
         <is>
           <t>Tăng tiêu hóa;Cân bằng hệ vi sinh;Tăng trưởng</t>
+        </is>
+      </c>
+      <c r="Z4" t="inlineStr">
+        <is>
+          <t>n</t>
         </is>
       </c>
     </row>
@@ -986,78 +925,74 @@
   </sheetPr>
   <dimension ref="A1:B7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="10" customWidth="1" min="1" max="1"/>
-    <col width="30" customWidth="1" min="2" max="2"/>
-  </cols>
   <sheetData>
-    <row r="1" ht="25" customHeight="1">
-      <c r="A1" s="3" t="inlineStr">
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>id</t>
         </is>
       </c>
-      <c r="B1" s="3" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>name</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="4" t="n">
+      <c r="A2" t="n">
         <v>1</v>
       </c>
-      <c r="B2" s="4" t="inlineStr">
+      <c r="B2" t="inlineStr">
         <is>
           <t>Thuốc Thú Cưng</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="4" t="n">
+      <c r="A3" t="n">
         <v>2</v>
       </c>
-      <c r="B3" s="4" t="inlineStr">
+      <c r="B3" t="inlineStr">
         <is>
           <t>Thuốc Gia Súc</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="4" t="n">
+      <c r="A4" t="n">
         <v>3</v>
       </c>
-      <c r="B4" s="4" t="inlineStr">
+      <c r="B4" t="inlineStr">
         <is>
           <t>Chế Phẩm Sinh Học</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="4" t="n">
+      <c r="A5" t="n">
         <v>4</v>
       </c>
-      <c r="B5" s="4" t="inlineStr">
+      <c r="B5" t="inlineStr">
         <is>
           <t>Vitamin &amp; Thực Phẩm Chức Năng</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="4" t="n">
+      <c r="A6" t="n">
         <v>5</v>
       </c>
-      <c r="B6" s="4" t="inlineStr">
+      <c r="B6" t="inlineStr">
         <is>
           <t>Thiết Bị Y Tế</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="4" t="n">
+      <c r="A7" t="n">
         <v>6</v>
       </c>
-      <c r="B7" s="4" t="inlineStr">
+      <c r="B7" t="inlineStr">
         <is>
           <t>Gia Cầm</t>
         </is>
@@ -1076,138 +1011,144 @@
   </sheetPr>
   <dimension ref="A1:A22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="50" customWidth="1" min="1" max="1"/>
-  </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="5" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>HƯỚNG DẪN SỬ DỤNG FILE EXCEL</t>
         </is>
       </c>
     </row>
+    <row r="2">
+      <c r="A2" t="inlineStr"/>
+    </row>
     <row r="3">
-      <c r="A3" s="2" t="inlineStr">
+      <c r="A3" t="inlineStr">
         <is>
           <t>SHEET "Products" (Sản phẩm):</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="2" t="inlineStr">
+      <c r="A4" t="inlineStr">
         <is>
           <t>Các cột cần thiết (*)</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="6" t="inlineStr">
+      <c r="A5" t="inlineStr">
         <is>
           <t>- id: Mã sản phẩm (bắt buộc)</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="6" t="inlineStr">
+      <c r="A6" t="inlineStr">
         <is>
           <t>- name: Tên sản phẩm (bắt buộc)</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="6" t="inlineStr">
+      <c r="A7" t="inlineStr">
         <is>
           <t>- category: Danh mục</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="6" t="inlineStr">
+      <c r="A8" t="inlineStr">
         <is>
           <t>- price: Giá bán</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="6" t="inlineStr">
+      <c r="A9" t="inlineStr">
         <is>
           <t>- description: Mô tả ngắn</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="6" t="inlineStr">
+      <c r="A10" t="inlineStr">
         <is>
           <t>- inStock: TRUE/FALSE (Còn hàng)</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="6" t="inlineStr">
+      <c r="A11" t="inlineStr">
         <is>
           <t>- featured: TRUE/FALSE (Sản phẩm nổi bật)</t>
         </is>
       </c>
     </row>
+    <row r="12">
+      <c r="A12" t="inlineStr"/>
+    </row>
     <row r="13">
-      <c r="A13" s="2" t="inlineStr">
+      <c r="A13" t="inlineStr">
         <is>
           <t>SHEET "Categories" (Danh mục):</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="6" t="inlineStr">
+      <c r="A14" t="inlineStr">
         <is>
           <t>- id: ID danh mục</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="6" t="inlineStr">
+      <c r="A15" t="inlineStr">
         <is>
           <t>- name: Tên danh mục</t>
         </is>
       </c>
     </row>
+    <row r="16">
+      <c r="A16" t="inlineStr"/>
+    </row>
     <row r="17">
-      <c r="A17" s="2" t="inlineStr">
+      <c r="A17" t="inlineStr">
         <is>
           <t>GHI CHÚ:</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="6" t="inlineStr">
+      <c r="A18" t="inlineStr">
         <is>
           <t>1. Cột "id" phải có giá trị duy nhất</t>
         </is>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="6" t="inlineStr">
+      <c r="A19" t="inlineStr">
         <is>
           <t>2. Sử dụng TRUE hoặc FALSE (in hoa) cho giá trị boolean</t>
         </is>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="6" t="inlineStr">
+      <c r="A20" t="inlineStr">
         <is>
           <t>3. Tên sheet phải chính xác: "Products", "Categories"</t>
         </is>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="6" t="inlineStr">
+      <c r="A21" t="inlineStr">
         <is>
           <t>4. File phải lưu ở: public/data/tamvet_product.xlsx</t>
         </is>
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="6" t="inlineStr">
+      <c r="A22" t="inlineStr">
         <is>
           <t>5. Định dạng: .xlsx (Excel 2007+)</t>
         </is>

</xml_diff>

<commit_message>
Update Tam Vet san pham 1
</commit_message>
<xml_diff>
--- a/public/data/tamvet_product.xlsx
+++ b/public/data/tamvet_product.xlsx
@@ -1,15 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Products" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Categories" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Hướng Dẫn" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Products" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Categories" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Hướng Dẫn" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -427,7 +427,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Z4"/>
+  <dimension ref="A1:Z3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -565,57 +565,57 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>TAMVET001</t>
+          <t>TAMVET002</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Thuốc Kháng Sinh Amoxicillin 500mg 2</t>
+          <t>Vitamin B Complex Cho Gia Súc</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Thuốc Thú Cưng</t>
+          <t>Vitamin &amp; Thực Phẩm Chức Năng</t>
         </is>
       </c>
       <c r="D2" t="n">
-        <v>45000</v>
+        <v>65000</v>
       </c>
       <c r="E2" t="n">
-        <v>50000</v>
+        <v>75000</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>Thuốc kháng sinh hiệu quả điều trị các bệnh nhiễm khuẩn</t>
+          <t>Bổ sung vitamin B giúp tăng sức đề kháng cho gia súc</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>Amoxicillin 500mg là thuốc kháng sinh beta-lactam có hiệu quả cao trong điều trị các bệnh nhiễm khuẩn ở động vật.&lt;div&gt;&lt;b&gt;Kiểm tra chi tiết sản phẩm&lt;/b&gt;&lt;/div&gt;</t>
+          <t>Vitamin B Complex là một sản phẩm bổ sung vitamin nhóm B toàn diện, giúp cải thiện sức khỏe tổng thể.</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>/images/tamvet-85766dd7-1765992017.jpg</t>
+          <t>/images/products/vitamin-b.jpg</t>
         </is>
       </c>
       <c r="I2" t="b">
         <v>1</v>
       </c>
       <c r="J2" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>10 vỉ/hộp</t>
+          <t>100ml/chai</t>
         </is>
       </c>
       <c r="L2" t="n">
-        <v>150</v>
+        <v>200</v>
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>Chó, Mèo, Gia súc</t>
+          <t>Gia súc</t>
         </is>
       </c>
       <c r="N2" t="inlineStr">
@@ -630,106 +630,110 @@
       </c>
       <c r="P2" t="inlineStr">
         <is>
-          <t>VN123456</t>
+          <t>VN123457</t>
         </is>
       </c>
       <c r="Q2" t="inlineStr">
         <is>
-          <t>Amoxicillin trihydrate 500mg</t>
+          <t>Thiamine,Riboflavin,Niacin,Pyridoxine</t>
         </is>
       </c>
       <c r="R2" t="inlineStr">
         <is>
-          <t>Chó: 20-40mg/kg, Mèo: 15-25mg/kg</t>
+          <t>5-10ml/ngày/đầu gia súc</t>
         </is>
       </c>
       <c r="S2" t="inlineStr">
         <is>
-          <t>Uống sau ăn 2-3 lần/ngày</t>
+          <t>Trộn vào thức ăn hoặc cho uống trực tiếp</t>
         </is>
       </c>
       <c r="T2" t="inlineStr">
         <is>
-          <t>Không sử dụng với thú có dị ứng penicillin</t>
+          <t>Bảo quản trong nơi mát mẻ, tránh ánh sáng</t>
         </is>
       </c>
       <c r="U2" t="inlineStr">
         <is>
-          <t>Bảo quản nơi khô ráo, nhiệt độ 15-25°C</t>
+          <t>Bảo quản ở 2-8°C</t>
         </is>
       </c>
       <c r="V2" t="n">
-        <v>4.5</v>
+        <v>4.2</v>
       </c>
       <c r="W2" t="n">
-        <v>32</v>
+        <v>18</v>
       </c>
       <c r="X2" t="inlineStr">
         <is>
-          <t>kháng sinh;nhiễm khuẩn;chó;mèo</t>
+          <t>vitamin;bổ sung;gia súc</t>
         </is>
       </c>
       <c r="Y2" t="inlineStr">
         <is>
-          <t>Kháng khuẩn;Diệt vi khuẩn</t>
-        </is>
-      </c>
-      <c r="Z2" t="inlineStr"/>
+          <t>Tăng sức đề kháng;Cải thiện sức khỏe</t>
+        </is>
+      </c>
+      <c r="Z2" t="inlineStr">
+        <is>
+          <t>n</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>TAMVET002</t>
+          <t>TAMVET003</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Vitamin B Complex Cho Gia Súc</t>
+          <t>Chế Phẩm Vi Sinh Tăng Tiêu Hóa</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Vitamin &amp; Thực Phẩm Chức Năng</t>
+          <t>Chế Phẩm Sinh Học</t>
         </is>
       </c>
       <c r="D3" t="n">
-        <v>65000</v>
+        <v>85000</v>
       </c>
       <c r="E3" t="n">
-        <v>75000</v>
+        <v>95000</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Bổ sung vitamin B giúp tăng sức đề kháng cho gia súc</t>
+          <t>Chế phẩm vi sinh giúp cân bằng hệ tiêu hóa</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>Vitamin B Complex là một sản phẩm bổ sung vitamin nhóm B toàn diện, giúp cải thiện sức khỏe tổng thể.</t>
+          <t>Chế phẩm này chứa các chủng vi sinh lợi ích giúp cân bằng hệ vi sinh đường ruột.</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>/images/products/vitamin-b.jpg</t>
+          <t>/images/products/probiotic.jpg</t>
         </is>
       </c>
       <c r="I3" t="b">
         <v>1</v>
       </c>
       <c r="J3" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>100ml/chai</t>
+          <t>500g/kg</t>
         </is>
       </c>
       <c r="L3" t="n">
-        <v>200</v>
+        <v>120</v>
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>Gia súc</t>
+          <t>Gia cầm, Gia súc, Cá</t>
         </is>
       </c>
       <c r="N3" t="inlineStr">
@@ -744,169 +748,51 @@
       </c>
       <c r="P3" t="inlineStr">
         <is>
-          <t>VN123457</t>
+          <t>VN123458</t>
         </is>
       </c>
       <c r="Q3" t="inlineStr">
         <is>
-          <t>Thiamine,Riboflavin,Niacin,Pyridoxine</t>
+          <t>Bacillus subtilis,Lactobacillus,Bifidobacterium</t>
         </is>
       </c>
       <c r="R3" t="inlineStr">
         <is>
-          <t>5-10ml/ngày/đầu gia súc</t>
+          <t>5-10g/tấn thức ăn</t>
         </is>
       </c>
       <c r="S3" t="inlineStr">
         <is>
-          <t>Trộn vào thức ăn hoặc cho uống trực tiếp</t>
+          <t>Trộn đều vào thức ăn tươi</t>
         </is>
       </c>
       <c r="T3" t="inlineStr">
         <is>
-          <t>Bảo quản trong nơi mát mẻ, tránh ánh sáng</t>
+          <t>Bảo quản ở nhiệt độ thấp, tránh ẩm ướt</t>
         </is>
       </c>
       <c r="U3" t="inlineStr">
         <is>
-          <t>Bảo quản ở 2-8°C</t>
+          <t>Bảo quản ở 2-8°C hoặc -18°C</t>
         </is>
       </c>
       <c r="V3" t="n">
-        <v>4.2</v>
+        <v>4.8</v>
       </c>
       <c r="W3" t="n">
-        <v>18</v>
+        <v>45</v>
       </c>
       <c r="X3" t="inlineStr">
         <is>
-          <t>vitamin;bổ sung;gia súc</t>
+          <t>vi sinh;tiêu hóa;chế phẩm</t>
         </is>
       </c>
       <c r="Y3" t="inlineStr">
         <is>
-          <t>Tăng sức đề kháng;Cải thiện sức khỏe</t>
+          <t>Tăng tiêu hóa;Cân bằng hệ vi sinh;Tăng trưởng</t>
         </is>
       </c>
       <c r="Z3" t="inlineStr">
-        <is>
-          <t>n</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>TAMVET003</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>Chế Phẩm Vi Sinh Tăng Tiêu Hóa</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>Chế Phẩm Sinh Học</t>
-        </is>
-      </c>
-      <c r="D4" t="n">
-        <v>85000</v>
-      </c>
-      <c r="E4" t="n">
-        <v>95000</v>
-      </c>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t>Chế phẩm vi sinh giúp cân bằng hệ tiêu hóa</t>
-        </is>
-      </c>
-      <c r="G4" t="inlineStr">
-        <is>
-          <t>Chế phẩm này chứa các chủng vi sinh lợi ích giúp cân bằng hệ vi sinh đường ruột.</t>
-        </is>
-      </c>
-      <c r="H4" t="inlineStr">
-        <is>
-          <t>/images/products/probiotic.jpg</t>
-        </is>
-      </c>
-      <c r="I4" t="b">
-        <v>1</v>
-      </c>
-      <c r="J4" t="b">
-        <v>1</v>
-      </c>
-      <c r="K4" t="inlineStr">
-        <is>
-          <t>500g/kg</t>
-        </is>
-      </c>
-      <c r="L4" t="n">
-        <v>120</v>
-      </c>
-      <c r="M4" t="inlineStr">
-        <is>
-          <t>Gia cầm, Gia súc, Cá</t>
-        </is>
-      </c>
-      <c r="N4" t="inlineStr">
-        <is>
-          <t>Tâm Vet</t>
-        </is>
-      </c>
-      <c r="O4" t="inlineStr">
-        <is>
-          <t>Việt Nam</t>
-        </is>
-      </c>
-      <c r="P4" t="inlineStr">
-        <is>
-          <t>VN123458</t>
-        </is>
-      </c>
-      <c r="Q4" t="inlineStr">
-        <is>
-          <t>Bacillus subtilis,Lactobacillus,Bifidobacterium</t>
-        </is>
-      </c>
-      <c r="R4" t="inlineStr">
-        <is>
-          <t>5-10g/tấn thức ăn</t>
-        </is>
-      </c>
-      <c r="S4" t="inlineStr">
-        <is>
-          <t>Trộn đều vào thức ăn tươi</t>
-        </is>
-      </c>
-      <c r="T4" t="inlineStr">
-        <is>
-          <t>Bảo quản ở nhiệt độ thấp, tránh ẩm ướt</t>
-        </is>
-      </c>
-      <c r="U4" t="inlineStr">
-        <is>
-          <t>Bảo quản ở 2-8°C hoặc -18°C</t>
-        </is>
-      </c>
-      <c r="V4" t="n">
-        <v>4.8</v>
-      </c>
-      <c r="W4" t="n">
-        <v>45</v>
-      </c>
-      <c r="X4" t="inlineStr">
-        <is>
-          <t>vi sinh;tiêu hóa;chế phẩm</t>
-        </is>
-      </c>
-      <c r="Y4" t="inlineStr">
-        <is>
-          <t>Tăng tiêu hóa;Cân bằng hệ vi sinh;Tăng trưởng</t>
-        </is>
-      </c>
-      <c r="Z4" t="inlineStr">
         <is>
           <t>n</t>
         </is>

</xml_diff>